<commit_message>
webscrapping working fine but two
</commit_message>
<xml_diff>
--- a/trial_Scraped.xlsx
+++ b/trial_Scraped.xlsx
@@ -519,11 +519,7 @@
           <t>http://www.digitalzentrum-berlin.de</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>manufacturing and processing, energy, health care, smart city, public administration, education, environment, transport &amp; mobility, automotive, agricultural biotechnology and food biotechnology</t>
-        </is>
-      </c>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Innovation management - 4, Knowledge transfer - 5, Sme Business Development - 5, SME support - 5, Technological innovation - 4, Technology transfer - 5</t>
@@ -574,11 +570,7 @@
           <t>https://www.handwerkdigital.de/</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>manufacturing and processing, energy, health care, smart city, public administration, education, environment, transport &amp; mobility, automotive, agricultural biotechnology and food biotechnology</t>
-        </is>
-      </c>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Technology transfer - 5</t>
@@ -680,11 +672,7 @@
           <t>https://idele.fr/</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>manufacturing and processing, energy, health care, smart city, public administration, education, environment, transport &amp; mobility, automotive, agricultural biotechnology and food biotechnology</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Field trial - 5, Knowledge transfer - 5, Prototyping - 3</t>
@@ -739,11 +727,7 @@
           <t>https://c-hub.pt</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>manufacturing and processing, energy, health care, smart city, public administration, education, environment, transport &amp; mobility, automotive, agricultural biotechnology and food biotechnology</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>Technological innovation - 5, Innovation management - 5, Public sector innovation - 5, Sme Business Development - 5, Technology transfer - 4</t>
@@ -804,11 +788,7 @@
           <t>Innovation management - 4, Prototyping - 4, Regional development - 5, SME support - 5, Sme Business Development - 4, Technology transfer - 3, Technological innovation - 3</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>artificial intelligence &amp; decision support, internet of things, cybersecurity, big data, digital twins, robotics, high performance computing, virtual reality, sensors &amp; vision processing systems, simulation engineering and modelling</t>
-        </is>
-      </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -970,11 +950,7 @@
           <t>Technological innovation - 4, Innovation management - 4, Prototyping - 4, Field trial - 3, Public sector innovation - 5, Sme Business Development - 5</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>artificial intelligence &amp; decision support, internet of things, cybersecurity, big data, digital twins, robotics, high performance computing, virtual reality, sensors &amp; vision processing systems, simulation engineering and modelling</t>
-        </is>
-      </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1015,16 +991,8 @@
           <t>https://aire-edih.eu/</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>manufacturing and processing, energy, health care, smart city, public administration, education, environment, transport &amp; mobility, automotive, agricultural biotechnology and food biotechnology</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>sme support, technological innovation, knowledge transfer, ecosystem building, technology transfer, innovation management, prototyping, sme business development, public sector innovation, finance</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>Artificial Intelligence &amp; Decision support - 5, Robotics - 5, Big data - 3, BI tools - 3, data - 5, Digital twins - 3, Cybersecurity - 3, Internet of Things - 3, Laser-based manufacturing and materials processing - 3, Logistics - 3, Sensors &amp; Vision Processing Systems - 3, Simulation engineering and modelling - 4, Mobility - 3, Virtual Reality - 3, Cloud Services - 3, Chemical engineering (plants, products) - 3, Cyber-physical systems - 3, High performance computing - 3, Software Architectures - 3, Human computer interaction - 5, Industrial biotechnology - 3, Communication network - 3, Organic and large area electronics - 3, Displays - 3</t>

</xml_diff>